<commit_message>
Sheet build: Charles Quaye as sole manager, no example row, new live link
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01QJ3FoxMD9ohKENf4AT4yHa
</commit_message>
<xml_diff>
--- a/group_contribution_tracker/google_sheet/ledger.xlsx
+++ b/group_contribution_tracker/google_sheet/ledger.xlsx
@@ -595,7 +595,7 @@
     <row r="4">
       <c r="A4" s="4" t="inlineStr">
         <is>
-          <t>Managed by Charles Quaye and Emmanuel Kpakpoe Addo. Members can view this sheet but not change it.</t>
+          <t>Managed by Charles Quaye. Members can view this sheet but not change it.</t>
         </is>
       </c>
     </row>
@@ -2233,7 +2233,7 @@
     <row r="5">
       <c r="A5" s="23" t="inlineStr">
         <is>
-          <t>MANAGERS (Charles Quaye, Emmanuel Kpakpoe Addo): open the Contributions tab and type one row per payment received:</t>
+          <t>MANAGER (Charles Quaye): open the Contributions tab and type one row per payment received:</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Sheet build: banner telling the manager where to type, carry-over of the first entry
Charles typed his first payment into the Ledger totals row instead of the
Contributions tab, which overwrote the SUM/COUNTIF formulas. The rebuilt
workbook puts a yellow banner in row 1 of the Ledger pointing him to the
Contributions tab, and build.py accepts a PREFILL variable so existing
payments can be carried into a fresh copy. README points at the new live
sheet.

Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01QJ3FoxMD9ohKENf4AT4yHa
</commit_message>
<xml_diff>
--- a/group_contribution_tracker/google_sheet/ledger.xlsx
+++ b/group_contribution_tracker/google_sheet/ledger.xlsx
@@ -22,7 +22,7 @@
     <numFmt numFmtId="164" formatCode="&quot;GH₵&quot;#,##0.00"/>
     <numFmt numFmtId="165" formatCode="d mmm yyyy"/>
   </numFmts>
-  <fonts count="15">
+  <fonts count="16">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -33,8 +33,8 @@
     <font>
       <name val="Arial"/>
       <b val="1"/>
-      <color rgb="001F6F50"/>
-      <sz val="9"/>
+      <color rgb="006D4F05"/>
+      <sz val="11"/>
     </font>
     <font>
       <name val="Arial"/>
@@ -78,6 +78,12 @@
     <font>
       <name val="Arial"/>
       <b val="1"/>
+      <color rgb="001F6F50"/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
       <color rgb="00FFFFFF"/>
       <sz val="10"/>
     </font>
@@ -107,12 +113,17 @@
       <sz val="10"/>
     </font>
   </fonts>
-  <fills count="5">
+  <fills count="6">
     <fill>
       <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FBF0D3"/>
+      </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
@@ -147,9 +158,11 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="24">
+  <cellXfs count="25">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
@@ -157,43 +170,44 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="164" fontId="6" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="6" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="1" fontId="7" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="1" fontId="7" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="9" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="8" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="10" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="10" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="164" fontId="10" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="164" fontId="11" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="9" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="10" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="165" fontId="12" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="12" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="164" fontId="12" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="165" fontId="13" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="13" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="13" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment wrapText="1"/>
     </xf>
   </cellXfs>
@@ -571,10 +585,10 @@
     <col width="4" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
-    <row r="1">
+    <row r="1" ht="34" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>CONTRIBUTION LEDGER</t>
+          <t>CHARLES: to record a payment, tap the 'Contributions' tab at the bottom of the screen. Do not type on this page.</t>
         </is>
       </c>
     </row>
@@ -648,29 +662,29 @@
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="1" t="inlineStr">
+      <c r="A10" s="10" t="inlineStr">
         <is>
           <t>BY MEMBER</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="10" t="inlineStr">
+      <c r="A11" s="11" t="inlineStr">
         <is>
           <t>#</t>
         </is>
       </c>
-      <c r="B11" s="10" t="inlineStr">
+      <c r="B11" s="11" t="inlineStr">
         <is>
           <t>Member</t>
         </is>
       </c>
-      <c r="C11" s="11" t="inlineStr">
+      <c r="C11" s="12" t="inlineStr">
         <is>
           <t>Payments</t>
         </is>
       </c>
-      <c r="D11" s="11" t="inlineStr">
+      <c r="D11" s="12" t="inlineStr">
         <is>
           <t>Total given</t>
         </is>
@@ -689,7 +703,7 @@
         <f>IF(B12="","",COUNTIF(Contributions!$B$2:$B$2000,B12))</f>
         <v/>
       </c>
-      <c r="D12" s="12">
+      <c r="D12" s="13">
         <f>IF(B12="","",SUMIF(Contributions!$B$2:$B$2000,B12,Contributions!$C$2:$C$2000))</f>
         <v/>
       </c>
@@ -707,7 +721,7 @@
         <f>IF(B13="","",COUNTIF(Contributions!$B$2:$B$2000,B13))</f>
         <v/>
       </c>
-      <c r="D13" s="12">
+      <c r="D13" s="13">
         <f>IF(B13="","",SUMIF(Contributions!$B$2:$B$2000,B13,Contributions!$C$2:$C$2000))</f>
         <v/>
       </c>
@@ -725,7 +739,7 @@
         <f>IF(B14="","",COUNTIF(Contributions!$B$2:$B$2000,B14))</f>
         <v/>
       </c>
-      <c r="D14" s="12">
+      <c r="D14" s="13">
         <f>IF(B14="","",SUMIF(Contributions!$B$2:$B$2000,B14,Contributions!$C$2:$C$2000))</f>
         <v/>
       </c>
@@ -743,7 +757,7 @@
         <f>IF(B15="","",COUNTIF(Contributions!$B$2:$B$2000,B15))</f>
         <v/>
       </c>
-      <c r="D15" s="12">
+      <c r="D15" s="13">
         <f>IF(B15="","",SUMIF(Contributions!$B$2:$B$2000,B15,Contributions!$C$2:$C$2000))</f>
         <v/>
       </c>
@@ -761,7 +775,7 @@
         <f>IF(B16="","",COUNTIF(Contributions!$B$2:$B$2000,B16))</f>
         <v/>
       </c>
-      <c r="D16" s="12">
+      <c r="D16" s="13">
         <f>IF(B16="","",SUMIF(Contributions!$B$2:$B$2000,B16,Contributions!$C$2:$C$2000))</f>
         <v/>
       </c>
@@ -779,7 +793,7 @@
         <f>IF(B17="","",COUNTIF(Contributions!$B$2:$B$2000,B17))</f>
         <v/>
       </c>
-      <c r="D17" s="12">
+      <c r="D17" s="13">
         <f>IF(B17="","",SUMIF(Contributions!$B$2:$B$2000,B17,Contributions!$C$2:$C$2000))</f>
         <v/>
       </c>
@@ -797,7 +811,7 @@
         <f>IF(B18="","",COUNTIF(Contributions!$B$2:$B$2000,B18))</f>
         <v/>
       </c>
-      <c r="D18" s="12">
+      <c r="D18" s="13">
         <f>IF(B18="","",SUMIF(Contributions!$B$2:$B$2000,B18,Contributions!$C$2:$C$2000))</f>
         <v/>
       </c>
@@ -815,7 +829,7 @@
         <f>IF(B19="","",COUNTIF(Contributions!$B$2:$B$2000,B19))</f>
         <v/>
       </c>
-      <c r="D19" s="12">
+      <c r="D19" s="13">
         <f>IF(B19="","",SUMIF(Contributions!$B$2:$B$2000,B19,Contributions!$C$2:$C$2000))</f>
         <v/>
       </c>
@@ -833,7 +847,7 @@
         <f>IF(B20="","",COUNTIF(Contributions!$B$2:$B$2000,B20))</f>
         <v/>
       </c>
-      <c r="D20" s="12">
+      <c r="D20" s="13">
         <f>IF(B20="","",SUMIF(Contributions!$B$2:$B$2000,B20,Contributions!$C$2:$C$2000))</f>
         <v/>
       </c>
@@ -851,7 +865,7 @@
         <f>IF(B21="","",COUNTIF(Contributions!$B$2:$B$2000,B21))</f>
         <v/>
       </c>
-      <c r="D21" s="12">
+      <c r="D21" s="13">
         <f>IF(B21="","",SUMIF(Contributions!$B$2:$B$2000,B21,Contributions!$C$2:$C$2000))</f>
         <v/>
       </c>
@@ -869,7 +883,7 @@
         <f>IF(B22="","",COUNTIF(Contributions!$B$2:$B$2000,B22))</f>
         <v/>
       </c>
-      <c r="D22" s="12">
+      <c r="D22" s="13">
         <f>IF(B22="","",SUMIF(Contributions!$B$2:$B$2000,B22,Contributions!$C$2:$C$2000))</f>
         <v/>
       </c>
@@ -887,7 +901,7 @@
         <f>IF(B23="","",COUNTIF(Contributions!$B$2:$B$2000,B23))</f>
         <v/>
       </c>
-      <c r="D23" s="12">
+      <c r="D23" s="13">
         <f>IF(B23="","",SUMIF(Contributions!$B$2:$B$2000,B23,Contributions!$C$2:$C$2000))</f>
         <v/>
       </c>
@@ -905,7 +919,7 @@
         <f>IF(B24="","",COUNTIF(Contributions!$B$2:$B$2000,B24))</f>
         <v/>
       </c>
-      <c r="D24" s="12">
+      <c r="D24" s="13">
         <f>IF(B24="","",SUMIF(Contributions!$B$2:$B$2000,B24,Contributions!$C$2:$C$2000))</f>
         <v/>
       </c>
@@ -923,7 +937,7 @@
         <f>IF(B25="","",COUNTIF(Contributions!$B$2:$B$2000,B25))</f>
         <v/>
       </c>
-      <c r="D25" s="12">
+      <c r="D25" s="13">
         <f>IF(B25="","",SUMIF(Contributions!$B$2:$B$2000,B25,Contributions!$C$2:$C$2000))</f>
         <v/>
       </c>
@@ -941,7 +955,7 @@
         <f>IF(B26="","",COUNTIF(Contributions!$B$2:$B$2000,B26))</f>
         <v/>
       </c>
-      <c r="D26" s="12">
+      <c r="D26" s="13">
         <f>IF(B26="","",SUMIF(Contributions!$B$2:$B$2000,B26,Contributions!$C$2:$C$2000))</f>
         <v/>
       </c>
@@ -959,7 +973,7 @@
         <f>IF(B27="","",COUNTIF(Contributions!$B$2:$B$2000,B27))</f>
         <v/>
       </c>
-      <c r="D27" s="12">
+      <c r="D27" s="13">
         <f>IF(B27="","",SUMIF(Contributions!$B$2:$B$2000,B27,Contributions!$C$2:$C$2000))</f>
         <v/>
       </c>
@@ -977,7 +991,7 @@
         <f>IF(B28="","",COUNTIF(Contributions!$B$2:$B$2000,B28))</f>
         <v/>
       </c>
-      <c r="D28" s="12">
+      <c r="D28" s="13">
         <f>IF(B28="","",SUMIF(Contributions!$B$2:$B$2000,B28,Contributions!$C$2:$C$2000))</f>
         <v/>
       </c>
@@ -995,7 +1009,7 @@
         <f>IF(B29="","",COUNTIF(Contributions!$B$2:$B$2000,B29))</f>
         <v/>
       </c>
-      <c r="D29" s="12">
+      <c r="D29" s="13">
         <f>IF(B29="","",SUMIF(Contributions!$B$2:$B$2000,B29,Contributions!$C$2:$C$2000))</f>
         <v/>
       </c>
@@ -1013,7 +1027,7 @@
         <f>IF(B30="","",COUNTIF(Contributions!$B$2:$B$2000,B30))</f>
         <v/>
       </c>
-      <c r="D30" s="12">
+      <c r="D30" s="13">
         <f>IF(B30="","",SUMIF(Contributions!$B$2:$B$2000,B30,Contributions!$C$2:$C$2000))</f>
         <v/>
       </c>
@@ -1031,7 +1045,7 @@
         <f>IF(B31="","",COUNTIF(Contributions!$B$2:$B$2000,B31))</f>
         <v/>
       </c>
-      <c r="D31" s="12">
+      <c r="D31" s="13">
         <f>IF(B31="","",SUMIF(Contributions!$B$2:$B$2000,B31,Contributions!$C$2:$C$2000))</f>
         <v/>
       </c>
@@ -1049,7 +1063,7 @@
         <f>IF(B32="","",COUNTIF(Contributions!$B$2:$B$2000,B32))</f>
         <v/>
       </c>
-      <c r="D32" s="12">
+      <c r="D32" s="13">
         <f>IF(B32="","",SUMIF(Contributions!$B$2:$B$2000,B32,Contributions!$C$2:$C$2000))</f>
         <v/>
       </c>
@@ -1067,7 +1081,7 @@
         <f>IF(B33="","",COUNTIF(Contributions!$B$2:$B$2000,B33))</f>
         <v/>
       </c>
-      <c r="D33" s="12">
+      <c r="D33" s="13">
         <f>IF(B33="","",SUMIF(Contributions!$B$2:$B$2000,B33,Contributions!$C$2:$C$2000))</f>
         <v/>
       </c>
@@ -1085,7 +1099,7 @@
         <f>IF(B34="","",COUNTIF(Contributions!$B$2:$B$2000,B34))</f>
         <v/>
       </c>
-      <c r="D34" s="12">
+      <c r="D34" s="13">
         <f>IF(B34="","",SUMIF(Contributions!$B$2:$B$2000,B34,Contributions!$C$2:$C$2000))</f>
         <v/>
       </c>
@@ -1103,7 +1117,7 @@
         <f>IF(B35="","",COUNTIF(Contributions!$B$2:$B$2000,B35))</f>
         <v/>
       </c>
-      <c r="D35" s="12">
+      <c r="D35" s="13">
         <f>IF(B35="","",SUMIF(Contributions!$B$2:$B$2000,B35,Contributions!$C$2:$C$2000))</f>
         <v/>
       </c>
@@ -1121,7 +1135,7 @@
         <f>IF(B36="","",COUNTIF(Contributions!$B$2:$B$2000,B36))</f>
         <v/>
       </c>
-      <c r="D36" s="12">
+      <c r="D36" s="13">
         <f>IF(B36="","",SUMIF(Contributions!$B$2:$B$2000,B36,Contributions!$C$2:$C$2000))</f>
         <v/>
       </c>
@@ -1139,7 +1153,7 @@
         <f>IF(B37="","",COUNTIF(Contributions!$B$2:$B$2000,B37))</f>
         <v/>
       </c>
-      <c r="D37" s="12">
+      <c r="D37" s="13">
         <f>IF(B37="","",SUMIF(Contributions!$B$2:$B$2000,B37,Contributions!$C$2:$C$2000))</f>
         <v/>
       </c>
@@ -1157,7 +1171,7 @@
         <f>IF(B38="","",COUNTIF(Contributions!$B$2:$B$2000,B38))</f>
         <v/>
       </c>
-      <c r="D38" s="12">
+      <c r="D38" s="13">
         <f>IF(B38="","",SUMIF(Contributions!$B$2:$B$2000,B38,Contributions!$C$2:$C$2000))</f>
         <v/>
       </c>
@@ -1175,7 +1189,7 @@
         <f>IF(B39="","",COUNTIF(Contributions!$B$2:$B$2000,B39))</f>
         <v/>
       </c>
-      <c r="D39" s="12">
+      <c r="D39" s="13">
         <f>IF(B39="","",SUMIF(Contributions!$B$2:$B$2000,B39,Contributions!$C$2:$C$2000))</f>
         <v/>
       </c>
@@ -1193,7 +1207,7 @@
         <f>IF(B40="","",COUNTIF(Contributions!$B$2:$B$2000,B40))</f>
         <v/>
       </c>
-      <c r="D40" s="12">
+      <c r="D40" s="13">
         <f>IF(B40="","",SUMIF(Contributions!$B$2:$B$2000,B40,Contributions!$C$2:$C$2000))</f>
         <v/>
       </c>
@@ -1211,7 +1225,7 @@
         <f>IF(B41="","",COUNTIF(Contributions!$B$2:$B$2000,B41))</f>
         <v/>
       </c>
-      <c r="D41" s="12">
+      <c r="D41" s="13">
         <f>IF(B41="","",SUMIF(Contributions!$B$2:$B$2000,B41,Contributions!$C$2:$C$2000))</f>
         <v/>
       </c>
@@ -1229,7 +1243,7 @@
         <f>IF(B42="","",COUNTIF(Contributions!$B$2:$B$2000,B42))</f>
         <v/>
       </c>
-      <c r="D42" s="12">
+      <c r="D42" s="13">
         <f>IF(B42="","",SUMIF(Contributions!$B$2:$B$2000,B42,Contributions!$C$2:$C$2000))</f>
         <v/>
       </c>
@@ -1247,7 +1261,7 @@
         <f>IF(B43="","",COUNTIF(Contributions!$B$2:$B$2000,B43))</f>
         <v/>
       </c>
-      <c r="D43" s="12">
+      <c r="D43" s="13">
         <f>IF(B43="","",SUMIF(Contributions!$B$2:$B$2000,B43,Contributions!$C$2:$C$2000))</f>
         <v/>
       </c>
@@ -1265,7 +1279,7 @@
         <f>IF(B44="","",COUNTIF(Contributions!$B$2:$B$2000,B44))</f>
         <v/>
       </c>
-      <c r="D44" s="12">
+      <c r="D44" s="13">
         <f>IF(B44="","",SUMIF(Contributions!$B$2:$B$2000,B44,Contributions!$C$2:$C$2000))</f>
         <v/>
       </c>
@@ -1283,7 +1297,7 @@
         <f>IF(B45="","",COUNTIF(Contributions!$B$2:$B$2000,B45))</f>
         <v/>
       </c>
-      <c r="D45" s="12">
+      <c r="D45" s="13">
         <f>IF(B45="","",SUMIF(Contributions!$B$2:$B$2000,B45,Contributions!$C$2:$C$2000))</f>
         <v/>
       </c>
@@ -1301,7 +1315,7 @@
         <f>IF(B46="","",COUNTIF(Contributions!$B$2:$B$2000,B46))</f>
         <v/>
       </c>
-      <c r="D46" s="12">
+      <c r="D46" s="13">
         <f>IF(B46="","",SUMIF(Contributions!$B$2:$B$2000,B46,Contributions!$C$2:$C$2000))</f>
         <v/>
       </c>
@@ -1319,7 +1333,7 @@
         <f>IF(B47="","",COUNTIF(Contributions!$B$2:$B$2000,B47))</f>
         <v/>
       </c>
-      <c r="D47" s="12">
+      <c r="D47" s="13">
         <f>IF(B47="","",SUMIF(Contributions!$B$2:$B$2000,B47,Contributions!$C$2:$C$2000))</f>
         <v/>
       </c>
@@ -1337,7 +1351,7 @@
         <f>IF(B48="","",COUNTIF(Contributions!$B$2:$B$2000,B48))</f>
         <v/>
       </c>
-      <c r="D48" s="12">
+      <c r="D48" s="13">
         <f>IF(B48="","",SUMIF(Contributions!$B$2:$B$2000,B48,Contributions!$C$2:$C$2000))</f>
         <v/>
       </c>
@@ -1355,7 +1369,7 @@
         <f>IF(B49="","",COUNTIF(Contributions!$B$2:$B$2000,B49))</f>
         <v/>
       </c>
-      <c r="D49" s="12">
+      <c r="D49" s="13">
         <f>IF(B49="","",SUMIF(Contributions!$B$2:$B$2000,B49,Contributions!$C$2:$C$2000))</f>
         <v/>
       </c>
@@ -1373,7 +1387,7 @@
         <f>IF(B50="","",COUNTIF(Contributions!$B$2:$B$2000,B50))</f>
         <v/>
       </c>
-      <c r="D50" s="12">
+      <c r="D50" s="13">
         <f>IF(B50="","",SUMIF(Contributions!$B$2:$B$2000,B50,Contributions!$C$2:$C$2000))</f>
         <v/>
       </c>
@@ -1391,7 +1405,7 @@
         <f>IF(B51="","",COUNTIF(Contributions!$B$2:$B$2000,B51))</f>
         <v/>
       </c>
-      <c r="D51" s="12">
+      <c r="D51" s="13">
         <f>IF(B51="","",SUMIF(Contributions!$B$2:$B$2000,B51,Contributions!$C$2:$C$2000))</f>
         <v/>
       </c>
@@ -1409,7 +1423,7 @@
         <f>IF(B52="","",COUNTIF(Contributions!$B$2:$B$2000,B52))</f>
         <v/>
       </c>
-      <c r="D52" s="12">
+      <c r="D52" s="13">
         <f>IF(B52="","",SUMIF(Contributions!$B$2:$B$2000,B52,Contributions!$C$2:$C$2000))</f>
         <v/>
       </c>
@@ -1427,7 +1441,7 @@
         <f>IF(B53="","",COUNTIF(Contributions!$B$2:$B$2000,B53))</f>
         <v/>
       </c>
-      <c r="D53" s="12">
+      <c r="D53" s="13">
         <f>IF(B53="","",SUMIF(Contributions!$B$2:$B$2000,B53,Contributions!$C$2:$C$2000))</f>
         <v/>
       </c>
@@ -1445,7 +1459,7 @@
         <f>IF(B54="","",COUNTIF(Contributions!$B$2:$B$2000,B54))</f>
         <v/>
       </c>
-      <c r="D54" s="12">
+      <c r="D54" s="13">
         <f>IF(B54="","",SUMIF(Contributions!$B$2:$B$2000,B54,Contributions!$C$2:$C$2000))</f>
         <v/>
       </c>
@@ -1463,7 +1477,7 @@
         <f>IF(B55="","",COUNTIF(Contributions!$B$2:$B$2000,B55))</f>
         <v/>
       </c>
-      <c r="D55" s="12">
+      <c r="D55" s="13">
         <f>IF(B55="","",SUMIF(Contributions!$B$2:$B$2000,B55,Contributions!$C$2:$C$2000))</f>
         <v/>
       </c>
@@ -1481,7 +1495,7 @@
         <f>IF(B56="","",COUNTIF(Contributions!$B$2:$B$2000,B56))</f>
         <v/>
       </c>
-      <c r="D56" s="12">
+      <c r="D56" s="13">
         <f>IF(B56="","",SUMIF(Contributions!$B$2:$B$2000,B56,Contributions!$C$2:$C$2000))</f>
         <v/>
       </c>
@@ -1499,7 +1513,7 @@
         <f>IF(B57="","",COUNTIF(Contributions!$B$2:$B$2000,B57))</f>
         <v/>
       </c>
-      <c r="D57" s="12">
+      <c r="D57" s="13">
         <f>IF(B57="","",SUMIF(Contributions!$B$2:$B$2000,B57,Contributions!$C$2:$C$2000))</f>
         <v/>
       </c>
@@ -1517,7 +1531,7 @@
         <f>IF(B58="","",COUNTIF(Contributions!$B$2:$B$2000,B58))</f>
         <v/>
       </c>
-      <c r="D58" s="12">
+      <c r="D58" s="13">
         <f>IF(B58="","",SUMIF(Contributions!$B$2:$B$2000,B58,Contributions!$C$2:$C$2000))</f>
         <v/>
       </c>
@@ -1535,7 +1549,7 @@
         <f>IF(B59="","",COUNTIF(Contributions!$B$2:$B$2000,B59))</f>
         <v/>
       </c>
-      <c r="D59" s="12">
+      <c r="D59" s="13">
         <f>IF(B59="","",SUMIF(Contributions!$B$2:$B$2000,B59,Contributions!$C$2:$C$2000))</f>
         <v/>
       </c>
@@ -1553,7 +1567,7 @@
         <f>IF(B60="","",COUNTIF(Contributions!$B$2:$B$2000,B60))</f>
         <v/>
       </c>
-      <c r="D60" s="12">
+      <c r="D60" s="13">
         <f>IF(B60="","",SUMIF(Contributions!$B$2:$B$2000,B60,Contributions!$C$2:$C$2000))</f>
         <v/>
       </c>
@@ -1571,7 +1585,7 @@
         <f>IF(B61="","",COUNTIF(Contributions!$B$2:$B$2000,B61))</f>
         <v/>
       </c>
-      <c r="D61" s="12">
+      <c r="D61" s="13">
         <f>IF(B61="","",SUMIF(Contributions!$B$2:$B$2000,B61,Contributions!$C$2:$C$2000))</f>
         <v/>
       </c>
@@ -1589,7 +1603,7 @@
         <f>IF(B62="","",COUNTIF(Contributions!$B$2:$B$2000,B62))</f>
         <v/>
       </c>
-      <c r="D62" s="12">
+      <c r="D62" s="13">
         <f>IF(B62="","",SUMIF(Contributions!$B$2:$B$2000,B62,Contributions!$C$2:$C$2000))</f>
         <v/>
       </c>
@@ -1607,7 +1621,7 @@
         <f>IF(B63="","",COUNTIF(Contributions!$B$2:$B$2000,B63))</f>
         <v/>
       </c>
-      <c r="D63" s="12">
+      <c r="D63" s="13">
         <f>IF(B63="","",SUMIF(Contributions!$B$2:$B$2000,B63,Contributions!$C$2:$C$2000))</f>
         <v/>
       </c>
@@ -1625,7 +1639,7 @@
         <f>IF(B64="","",COUNTIF(Contributions!$B$2:$B$2000,B64))</f>
         <v/>
       </c>
-      <c r="D64" s="12">
+      <c r="D64" s="13">
         <f>IF(B64="","",SUMIF(Contributions!$B$2:$B$2000,B64,Contributions!$C$2:$C$2000))</f>
         <v/>
       </c>
@@ -1643,7 +1657,7 @@
         <f>IF(B65="","",COUNTIF(Contributions!$B$2:$B$2000,B65))</f>
         <v/>
       </c>
-      <c r="D65" s="12">
+      <c r="D65" s="13">
         <f>IF(B65="","",SUMIF(Contributions!$B$2:$B$2000,B65,Contributions!$C$2:$C$2000))</f>
         <v/>
       </c>
@@ -1661,7 +1675,7 @@
         <f>IF(B66="","",COUNTIF(Contributions!$B$2:$B$2000,B66))</f>
         <v/>
       </c>
-      <c r="D66" s="12">
+      <c r="D66" s="13">
         <f>IF(B66="","",SUMIF(Contributions!$B$2:$B$2000,B66,Contributions!$C$2:$C$2000))</f>
         <v/>
       </c>
@@ -1679,7 +1693,7 @@
         <f>IF(B67="","",COUNTIF(Contributions!$B$2:$B$2000,B67))</f>
         <v/>
       </c>
-      <c r="D67" s="12">
+      <c r="D67" s="13">
         <f>IF(B67="","",SUMIF(Contributions!$B$2:$B$2000,B67,Contributions!$C$2:$C$2000))</f>
         <v/>
       </c>
@@ -1697,7 +1711,7 @@
         <f>IF(B68="","",COUNTIF(Contributions!$B$2:$B$2000,B68))</f>
         <v/>
       </c>
-      <c r="D68" s="12">
+      <c r="D68" s="13">
         <f>IF(B68="","",SUMIF(Contributions!$B$2:$B$2000,B68,Contributions!$C$2:$C$2000))</f>
         <v/>
       </c>
@@ -1715,7 +1729,7 @@
         <f>IF(B69="","",COUNTIF(Contributions!$B$2:$B$2000,B69))</f>
         <v/>
       </c>
-      <c r="D69" s="12">
+      <c r="D69" s="13">
         <f>IF(B69="","",SUMIF(Contributions!$B$2:$B$2000,B69,Contributions!$C$2:$C$2000))</f>
         <v/>
       </c>
@@ -1733,7 +1747,7 @@
         <f>IF(B70="","",COUNTIF(Contributions!$B$2:$B$2000,B70))</f>
         <v/>
       </c>
-      <c r="D70" s="12">
+      <c r="D70" s="13">
         <f>IF(B70="","",SUMIF(Contributions!$B$2:$B$2000,B70,Contributions!$C$2:$C$2000))</f>
         <v/>
       </c>
@@ -1751,27 +1765,27 @@
         <f>IF(B71="","",COUNTIF(Contributions!$B$2:$B$2000,B71))</f>
         <v/>
       </c>
-      <c r="D71" s="12">
+      <c r="D71" s="13">
         <f>IF(B71="","",SUMIF(Contributions!$B$2:$B$2000,B71,Contributions!$C$2:$C$2000))</f>
         <v/>
       </c>
     </row>
     <row r="72">
-      <c r="B72" s="13">
+      <c r="B72" s="14">
         <f>COUNTIF(B12:B71,"?*")&amp;" contributors"</f>
         <v/>
       </c>
-      <c r="C72" s="14">
+      <c r="C72" s="15">
         <f>SUM(C12:C71)</f>
         <v/>
       </c>
-      <c r="D72" s="15">
+      <c r="D72" s="16">
         <f>SUM(D12:D71)</f>
         <v/>
       </c>
     </row>
     <row r="74">
-      <c r="A74" s="16" t="inlineStr">
+      <c r="A74" s="17" t="inlineStr">
         <is>
           <t>Every payment, in date order, is on the Contributions tab. Only the managers can add or change entries.</t>
         </is>
@@ -1779,7 +1793,8 @@
     </row>
   </sheetData>
   <sheetProtection selectLockedCells="0" selectUnlockedCells="0" sheet="1" objects="0" insertRows="1" insertHyperlinks="1" autoFilter="1" scenarios="0" formatColumns="1" deleteColumns="1" insertColumns="1" pivotTables="1" deleteRows="1" formatCells="1" formatRows="1" sort="1"/>
-  <mergeCells count="3">
+  <mergeCells count="4">
+    <mergeCell ref="A1:D1"/>
     <mergeCell ref="A4:D4"/>
     <mergeCell ref="A3:D3"/>
     <mergeCell ref="A2:D2"/>
@@ -1797,393 +1812,405 @@
   <dimension ref="A1:D61"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="14" customWidth="1" style="17" min="1" max="1"/>
+    <col width="14" customWidth="1" style="18" min="1" max="1"/>
     <col width="30" customWidth="1" min="2" max="2"/>
-    <col width="15" customWidth="1" style="12" min="3" max="3"/>
+    <col width="15" customWidth="1" style="13" min="3" max="3"/>
     <col width="40" customWidth="1" min="4" max="4"/>
   </cols>
   <sheetData>
     <row r="1" ht="24" customHeight="1">
-      <c r="A1" s="18" t="inlineStr">
+      <c r="A1" s="19" t="inlineStr">
         <is>
           <t>Date received</t>
         </is>
       </c>
-      <c r="B1" s="18" t="inlineStr">
+      <c r="B1" s="19" t="inlineStr">
         <is>
           <t>Member name</t>
         </is>
       </c>
-      <c r="C1" s="18" t="inlineStr">
+      <c r="C1" s="19" t="inlineStr">
         <is>
           <t>Amount (GHS)</t>
         </is>
       </c>
-      <c r="D1" s="18" t="inlineStr">
+      <c r="D1" s="19" t="inlineStr">
         <is>
           <t>Note (optional)</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="19" t="n"/>
-      <c r="B2" s="20" t="n"/>
-      <c r="C2" s="21" t="n"/>
-      <c r="D2" s="20" t="n"/>
+      <c r="A2" s="20" t="n">
+        <v>46281</v>
+      </c>
+      <c r="B2" s="21" t="inlineStr">
+        <is>
+          <t>Nii Nelson</t>
+        </is>
+      </c>
+      <c r="C2" s="22" t="n">
+        <v>100</v>
+      </c>
+      <c r="D2" s="21" t="inlineStr">
+        <is>
+          <t>Carried over from the first entry. Charles, correct the date if needed</t>
+        </is>
+      </c>
     </row>
     <row r="3">
-      <c r="A3" s="19" t="n"/>
-      <c r="B3" s="20" t="n"/>
-      <c r="C3" s="21" t="n"/>
-      <c r="D3" s="20" t="n"/>
+      <c r="A3" s="20" t="n"/>
+      <c r="B3" s="21" t="n"/>
+      <c r="C3" s="22" t="n"/>
+      <c r="D3" s="21" t="n"/>
     </row>
     <row r="4">
-      <c r="A4" s="19" t="n"/>
-      <c r="B4" s="20" t="n"/>
-      <c r="C4" s="21" t="n"/>
-      <c r="D4" s="20" t="n"/>
+      <c r="A4" s="20" t="n"/>
+      <c r="B4" s="21" t="n"/>
+      <c r="C4" s="22" t="n"/>
+      <c r="D4" s="21" t="n"/>
     </row>
     <row r="5">
-      <c r="A5" s="19" t="n"/>
-      <c r="B5" s="20" t="n"/>
-      <c r="C5" s="21" t="n"/>
-      <c r="D5" s="20" t="n"/>
+      <c r="A5" s="20" t="n"/>
+      <c r="B5" s="21" t="n"/>
+      <c r="C5" s="22" t="n"/>
+      <c r="D5" s="21" t="n"/>
     </row>
     <row r="6">
-      <c r="A6" s="19" t="n"/>
-      <c r="B6" s="20" t="n"/>
-      <c r="C6" s="21" t="n"/>
-      <c r="D6" s="20" t="n"/>
+      <c r="A6" s="20" t="n"/>
+      <c r="B6" s="21" t="n"/>
+      <c r="C6" s="22" t="n"/>
+      <c r="D6" s="21" t="n"/>
     </row>
     <row r="7">
-      <c r="A7" s="19" t="n"/>
-      <c r="B7" s="20" t="n"/>
-      <c r="C7" s="21" t="n"/>
-      <c r="D7" s="20" t="n"/>
+      <c r="A7" s="20" t="n"/>
+      <c r="B7" s="21" t="n"/>
+      <c r="C7" s="22" t="n"/>
+      <c r="D7" s="21" t="n"/>
     </row>
     <row r="8">
-      <c r="A8" s="19" t="n"/>
-      <c r="B8" s="20" t="n"/>
-      <c r="C8" s="21" t="n"/>
-      <c r="D8" s="20" t="n"/>
+      <c r="A8" s="20" t="n"/>
+      <c r="B8" s="21" t="n"/>
+      <c r="C8" s="22" t="n"/>
+      <c r="D8" s="21" t="n"/>
     </row>
     <row r="9">
-      <c r="A9" s="19" t="n"/>
-      <c r="B9" s="20" t="n"/>
-      <c r="C9" s="21" t="n"/>
-      <c r="D9" s="20" t="n"/>
+      <c r="A9" s="20" t="n"/>
+      <c r="B9" s="21" t="n"/>
+      <c r="C9" s="22" t="n"/>
+      <c r="D9" s="21" t="n"/>
     </row>
     <row r="10">
-      <c r="A10" s="19" t="n"/>
-      <c r="B10" s="20" t="n"/>
-      <c r="C10" s="21" t="n"/>
-      <c r="D10" s="20" t="n"/>
+      <c r="A10" s="20" t="n"/>
+      <c r="B10" s="21" t="n"/>
+      <c r="C10" s="22" t="n"/>
+      <c r="D10" s="21" t="n"/>
     </row>
     <row r="11">
-      <c r="A11" s="19" t="n"/>
-      <c r="B11" s="20" t="n"/>
-      <c r="C11" s="21" t="n"/>
-      <c r="D11" s="20" t="n"/>
+      <c r="A11" s="20" t="n"/>
+      <c r="B11" s="21" t="n"/>
+      <c r="C11" s="22" t="n"/>
+      <c r="D11" s="21" t="n"/>
     </row>
     <row r="12">
-      <c r="A12" s="19" t="n"/>
-      <c r="B12" s="20" t="n"/>
-      <c r="C12" s="21" t="n"/>
-      <c r="D12" s="20" t="n"/>
+      <c r="A12" s="20" t="n"/>
+      <c r="B12" s="21" t="n"/>
+      <c r="C12" s="22" t="n"/>
+      <c r="D12" s="21" t="n"/>
     </row>
     <row r="13">
-      <c r="A13" s="19" t="n"/>
-      <c r="B13" s="20" t="n"/>
-      <c r="C13" s="21" t="n"/>
-      <c r="D13" s="20" t="n"/>
+      <c r="A13" s="20" t="n"/>
+      <c r="B13" s="21" t="n"/>
+      <c r="C13" s="22" t="n"/>
+      <c r="D13" s="21" t="n"/>
     </row>
     <row r="14">
-      <c r="A14" s="19" t="n"/>
-      <c r="B14" s="20" t="n"/>
-      <c r="C14" s="21" t="n"/>
-      <c r="D14" s="20" t="n"/>
+      <c r="A14" s="20" t="n"/>
+      <c r="B14" s="21" t="n"/>
+      <c r="C14" s="22" t="n"/>
+      <c r="D14" s="21" t="n"/>
     </row>
     <row r="15">
-      <c r="A15" s="19" t="n"/>
-      <c r="B15" s="20" t="n"/>
-      <c r="C15" s="21" t="n"/>
-      <c r="D15" s="20" t="n"/>
+      <c r="A15" s="20" t="n"/>
+      <c r="B15" s="21" t="n"/>
+      <c r="C15" s="22" t="n"/>
+      <c r="D15" s="21" t="n"/>
     </row>
     <row r="16">
-      <c r="A16" s="19" t="n"/>
-      <c r="B16" s="20" t="n"/>
-      <c r="C16" s="21" t="n"/>
-      <c r="D16" s="20" t="n"/>
+      <c r="A16" s="20" t="n"/>
+      <c r="B16" s="21" t="n"/>
+      <c r="C16" s="22" t="n"/>
+      <c r="D16" s="21" t="n"/>
     </row>
     <row r="17">
-      <c r="A17" s="19" t="n"/>
-      <c r="B17" s="20" t="n"/>
-      <c r="C17" s="21" t="n"/>
-      <c r="D17" s="20" t="n"/>
+      <c r="A17" s="20" t="n"/>
+      <c r="B17" s="21" t="n"/>
+      <c r="C17" s="22" t="n"/>
+      <c r="D17" s="21" t="n"/>
     </row>
     <row r="18">
-      <c r="A18" s="19" t="n"/>
-      <c r="B18" s="20" t="n"/>
-      <c r="C18" s="21" t="n"/>
-      <c r="D18" s="20" t="n"/>
+      <c r="A18" s="20" t="n"/>
+      <c r="B18" s="21" t="n"/>
+      <c r="C18" s="22" t="n"/>
+      <c r="D18" s="21" t="n"/>
     </row>
     <row r="19">
-      <c r="A19" s="19" t="n"/>
-      <c r="B19" s="20" t="n"/>
-      <c r="C19" s="21" t="n"/>
-      <c r="D19" s="20" t="n"/>
+      <c r="A19" s="20" t="n"/>
+      <c r="B19" s="21" t="n"/>
+      <c r="C19" s="22" t="n"/>
+      <c r="D19" s="21" t="n"/>
     </row>
     <row r="20">
-      <c r="A20" s="19" t="n"/>
-      <c r="B20" s="20" t="n"/>
-      <c r="C20" s="21" t="n"/>
-      <c r="D20" s="20" t="n"/>
+      <c r="A20" s="20" t="n"/>
+      <c r="B20" s="21" t="n"/>
+      <c r="C20" s="22" t="n"/>
+      <c r="D20" s="21" t="n"/>
     </row>
     <row r="21">
-      <c r="A21" s="19" t="n"/>
-      <c r="B21" s="20" t="n"/>
-      <c r="C21" s="21" t="n"/>
-      <c r="D21" s="20" t="n"/>
+      <c r="A21" s="20" t="n"/>
+      <c r="B21" s="21" t="n"/>
+      <c r="C21" s="22" t="n"/>
+      <c r="D21" s="21" t="n"/>
     </row>
     <row r="22">
-      <c r="A22" s="19" t="n"/>
-      <c r="B22" s="20" t="n"/>
-      <c r="C22" s="21" t="n"/>
-      <c r="D22" s="20" t="n"/>
+      <c r="A22" s="20" t="n"/>
+      <c r="B22" s="21" t="n"/>
+      <c r="C22" s="22" t="n"/>
+      <c r="D22" s="21" t="n"/>
     </row>
     <row r="23">
-      <c r="A23" s="19" t="n"/>
-      <c r="B23" s="20" t="n"/>
-      <c r="C23" s="21" t="n"/>
-      <c r="D23" s="20" t="n"/>
+      <c r="A23" s="20" t="n"/>
+      <c r="B23" s="21" t="n"/>
+      <c r="C23" s="22" t="n"/>
+      <c r="D23" s="21" t="n"/>
     </row>
     <row r="24">
-      <c r="A24" s="19" t="n"/>
-      <c r="B24" s="20" t="n"/>
-      <c r="C24" s="21" t="n"/>
-      <c r="D24" s="20" t="n"/>
+      <c r="A24" s="20" t="n"/>
+      <c r="B24" s="21" t="n"/>
+      <c r="C24" s="22" t="n"/>
+      <c r="D24" s="21" t="n"/>
     </row>
     <row r="25">
-      <c r="A25" s="19" t="n"/>
-      <c r="B25" s="20" t="n"/>
-      <c r="C25" s="21" t="n"/>
-      <c r="D25" s="20" t="n"/>
+      <c r="A25" s="20" t="n"/>
+      <c r="B25" s="21" t="n"/>
+      <c r="C25" s="22" t="n"/>
+      <c r="D25" s="21" t="n"/>
     </row>
     <row r="26">
-      <c r="A26" s="19" t="n"/>
-      <c r="B26" s="20" t="n"/>
-      <c r="C26" s="21" t="n"/>
-      <c r="D26" s="20" t="n"/>
+      <c r="A26" s="20" t="n"/>
+      <c r="B26" s="21" t="n"/>
+      <c r="C26" s="22" t="n"/>
+      <c r="D26" s="21" t="n"/>
     </row>
     <row r="27">
-      <c r="A27" s="19" t="n"/>
-      <c r="B27" s="20" t="n"/>
-      <c r="C27" s="21" t="n"/>
-      <c r="D27" s="20" t="n"/>
+      <c r="A27" s="20" t="n"/>
+      <c r="B27" s="21" t="n"/>
+      <c r="C27" s="22" t="n"/>
+      <c r="D27" s="21" t="n"/>
     </row>
     <row r="28">
-      <c r="A28" s="19" t="n"/>
-      <c r="B28" s="20" t="n"/>
-      <c r="C28" s="21" t="n"/>
-      <c r="D28" s="20" t="n"/>
+      <c r="A28" s="20" t="n"/>
+      <c r="B28" s="21" t="n"/>
+      <c r="C28" s="22" t="n"/>
+      <c r="D28" s="21" t="n"/>
     </row>
     <row r="29">
-      <c r="A29" s="19" t="n"/>
-      <c r="B29" s="20" t="n"/>
-      <c r="C29" s="21" t="n"/>
-      <c r="D29" s="20" t="n"/>
+      <c r="A29" s="20" t="n"/>
+      <c r="B29" s="21" t="n"/>
+      <c r="C29" s="22" t="n"/>
+      <c r="D29" s="21" t="n"/>
     </row>
     <row r="30">
-      <c r="A30" s="19" t="n"/>
-      <c r="B30" s="20" t="n"/>
-      <c r="C30" s="21" t="n"/>
-      <c r="D30" s="20" t="n"/>
+      <c r="A30" s="20" t="n"/>
+      <c r="B30" s="21" t="n"/>
+      <c r="C30" s="22" t="n"/>
+      <c r="D30" s="21" t="n"/>
     </row>
     <row r="31">
-      <c r="A31" s="19" t="n"/>
-      <c r="B31" s="20" t="n"/>
-      <c r="C31" s="21" t="n"/>
-      <c r="D31" s="20" t="n"/>
+      <c r="A31" s="20" t="n"/>
+      <c r="B31" s="21" t="n"/>
+      <c r="C31" s="22" t="n"/>
+      <c r="D31" s="21" t="n"/>
     </row>
     <row r="32">
-      <c r="A32" s="19" t="n"/>
-      <c r="B32" s="20" t="n"/>
-      <c r="C32" s="21" t="n"/>
-      <c r="D32" s="20" t="n"/>
+      <c r="A32" s="20" t="n"/>
+      <c r="B32" s="21" t="n"/>
+      <c r="C32" s="22" t="n"/>
+      <c r="D32" s="21" t="n"/>
     </row>
     <row r="33">
-      <c r="A33" s="19" t="n"/>
-      <c r="B33" s="20" t="n"/>
-      <c r="C33" s="21" t="n"/>
-      <c r="D33" s="20" t="n"/>
+      <c r="A33" s="20" t="n"/>
+      <c r="B33" s="21" t="n"/>
+      <c r="C33" s="22" t="n"/>
+      <c r="D33" s="21" t="n"/>
     </row>
     <row r="34">
-      <c r="A34" s="19" t="n"/>
-      <c r="B34" s="20" t="n"/>
-      <c r="C34" s="21" t="n"/>
-      <c r="D34" s="20" t="n"/>
+      <c r="A34" s="20" t="n"/>
+      <c r="B34" s="21" t="n"/>
+      <c r="C34" s="22" t="n"/>
+      <c r="D34" s="21" t="n"/>
     </row>
     <row r="35">
-      <c r="A35" s="19" t="n"/>
-      <c r="B35" s="20" t="n"/>
-      <c r="C35" s="21" t="n"/>
-      <c r="D35" s="20" t="n"/>
+      <c r="A35" s="20" t="n"/>
+      <c r="B35" s="21" t="n"/>
+      <c r="C35" s="22" t="n"/>
+      <c r="D35" s="21" t="n"/>
     </row>
     <row r="36">
-      <c r="A36" s="19" t="n"/>
-      <c r="B36" s="20" t="n"/>
-      <c r="C36" s="21" t="n"/>
-      <c r="D36" s="20" t="n"/>
+      <c r="A36" s="20" t="n"/>
+      <c r="B36" s="21" t="n"/>
+      <c r="C36" s="22" t="n"/>
+      <c r="D36" s="21" t="n"/>
     </row>
     <row r="37">
-      <c r="A37" s="19" t="n"/>
-      <c r="B37" s="20" t="n"/>
-      <c r="C37" s="21" t="n"/>
-      <c r="D37" s="20" t="n"/>
+      <c r="A37" s="20" t="n"/>
+      <c r="B37" s="21" t="n"/>
+      <c r="C37" s="22" t="n"/>
+      <c r="D37" s="21" t="n"/>
     </row>
     <row r="38">
-      <c r="A38" s="19" t="n"/>
-      <c r="B38" s="20" t="n"/>
-      <c r="C38" s="21" t="n"/>
-      <c r="D38" s="20" t="n"/>
+      <c r="A38" s="20" t="n"/>
+      <c r="B38" s="21" t="n"/>
+      <c r="C38" s="22" t="n"/>
+      <c r="D38" s="21" t="n"/>
     </row>
     <row r="39">
-      <c r="A39" s="19" t="n"/>
-      <c r="B39" s="20" t="n"/>
-      <c r="C39" s="21" t="n"/>
-      <c r="D39" s="20" t="n"/>
+      <c r="A39" s="20" t="n"/>
+      <c r="B39" s="21" t="n"/>
+      <c r="C39" s="22" t="n"/>
+      <c r="D39" s="21" t="n"/>
     </row>
     <row r="40">
-      <c r="A40" s="19" t="n"/>
-      <c r="B40" s="20" t="n"/>
-      <c r="C40" s="21" t="n"/>
-      <c r="D40" s="20" t="n"/>
+      <c r="A40" s="20" t="n"/>
+      <c r="B40" s="21" t="n"/>
+      <c r="C40" s="22" t="n"/>
+      <c r="D40" s="21" t="n"/>
     </row>
     <row r="41">
-      <c r="A41" s="19" t="n"/>
-      <c r="B41" s="20" t="n"/>
-      <c r="C41" s="21" t="n"/>
-      <c r="D41" s="20" t="n"/>
+      <c r="A41" s="20" t="n"/>
+      <c r="B41" s="21" t="n"/>
+      <c r="C41" s="22" t="n"/>
+      <c r="D41" s="21" t="n"/>
     </row>
     <row r="42">
-      <c r="A42" s="19" t="n"/>
-      <c r="B42" s="20" t="n"/>
-      <c r="C42" s="21" t="n"/>
-      <c r="D42" s="20" t="n"/>
+      <c r="A42" s="20" t="n"/>
+      <c r="B42" s="21" t="n"/>
+      <c r="C42" s="22" t="n"/>
+      <c r="D42" s="21" t="n"/>
     </row>
     <row r="43">
-      <c r="A43" s="19" t="n"/>
-      <c r="B43" s="20" t="n"/>
-      <c r="C43" s="21" t="n"/>
-      <c r="D43" s="20" t="n"/>
+      <c r="A43" s="20" t="n"/>
+      <c r="B43" s="21" t="n"/>
+      <c r="C43" s="22" t="n"/>
+      <c r="D43" s="21" t="n"/>
     </row>
     <row r="44">
-      <c r="A44" s="19" t="n"/>
-      <c r="B44" s="20" t="n"/>
-      <c r="C44" s="21" t="n"/>
-      <c r="D44" s="20" t="n"/>
+      <c r="A44" s="20" t="n"/>
+      <c r="B44" s="21" t="n"/>
+      <c r="C44" s="22" t="n"/>
+      <c r="D44" s="21" t="n"/>
     </row>
     <row r="45">
-      <c r="A45" s="19" t="n"/>
-      <c r="B45" s="20" t="n"/>
-      <c r="C45" s="21" t="n"/>
-      <c r="D45" s="20" t="n"/>
+      <c r="A45" s="20" t="n"/>
+      <c r="B45" s="21" t="n"/>
+      <c r="C45" s="22" t="n"/>
+      <c r="D45" s="21" t="n"/>
     </row>
     <row r="46">
-      <c r="A46" s="19" t="n"/>
-      <c r="B46" s="20" t="n"/>
-      <c r="C46" s="21" t="n"/>
-      <c r="D46" s="20" t="n"/>
+      <c r="A46" s="20" t="n"/>
+      <c r="B46" s="21" t="n"/>
+      <c r="C46" s="22" t="n"/>
+      <c r="D46" s="21" t="n"/>
     </row>
     <row r="47">
-      <c r="A47" s="19" t="n"/>
-      <c r="B47" s="20" t="n"/>
-      <c r="C47" s="21" t="n"/>
-      <c r="D47" s="20" t="n"/>
+      <c r="A47" s="20" t="n"/>
+      <c r="B47" s="21" t="n"/>
+      <c r="C47" s="22" t="n"/>
+      <c r="D47" s="21" t="n"/>
     </row>
     <row r="48">
-      <c r="A48" s="19" t="n"/>
-      <c r="B48" s="20" t="n"/>
-      <c r="C48" s="21" t="n"/>
-      <c r="D48" s="20" t="n"/>
+      <c r="A48" s="20" t="n"/>
+      <c r="B48" s="21" t="n"/>
+      <c r="C48" s="22" t="n"/>
+      <c r="D48" s="21" t="n"/>
     </row>
     <row r="49">
-      <c r="A49" s="19" t="n"/>
-      <c r="B49" s="20" t="n"/>
-      <c r="C49" s="21" t="n"/>
-      <c r="D49" s="20" t="n"/>
+      <c r="A49" s="20" t="n"/>
+      <c r="B49" s="21" t="n"/>
+      <c r="C49" s="22" t="n"/>
+      <c r="D49" s="21" t="n"/>
     </row>
     <row r="50">
-      <c r="A50" s="19" t="n"/>
-      <c r="B50" s="20" t="n"/>
-      <c r="C50" s="21" t="n"/>
-      <c r="D50" s="20" t="n"/>
+      <c r="A50" s="20" t="n"/>
+      <c r="B50" s="21" t="n"/>
+      <c r="C50" s="22" t="n"/>
+      <c r="D50" s="21" t="n"/>
     </row>
     <row r="51">
-      <c r="A51" s="19" t="n"/>
-      <c r="B51" s="20" t="n"/>
-      <c r="C51" s="21" t="n"/>
-      <c r="D51" s="20" t="n"/>
+      <c r="A51" s="20" t="n"/>
+      <c r="B51" s="21" t="n"/>
+      <c r="C51" s="22" t="n"/>
+      <c r="D51" s="21" t="n"/>
     </row>
     <row r="52">
-      <c r="A52" s="19" t="n"/>
-      <c r="B52" s="20" t="n"/>
-      <c r="C52" s="21" t="n"/>
-      <c r="D52" s="20" t="n"/>
+      <c r="A52" s="20" t="n"/>
+      <c r="B52" s="21" t="n"/>
+      <c r="C52" s="22" t="n"/>
+      <c r="D52" s="21" t="n"/>
     </row>
     <row r="53">
-      <c r="A53" s="19" t="n"/>
-      <c r="B53" s="20" t="n"/>
-      <c r="C53" s="21" t="n"/>
-      <c r="D53" s="20" t="n"/>
+      <c r="A53" s="20" t="n"/>
+      <c r="B53" s="21" t="n"/>
+      <c r="C53" s="22" t="n"/>
+      <c r="D53" s="21" t="n"/>
     </row>
     <row r="54">
-      <c r="A54" s="19" t="n"/>
-      <c r="B54" s="20" t="n"/>
-      <c r="C54" s="21" t="n"/>
-      <c r="D54" s="20" t="n"/>
+      <c r="A54" s="20" t="n"/>
+      <c r="B54" s="21" t="n"/>
+      <c r="C54" s="22" t="n"/>
+      <c r="D54" s="21" t="n"/>
     </row>
     <row r="55">
-      <c r="A55" s="19" t="n"/>
-      <c r="B55" s="20" t="n"/>
-      <c r="C55" s="21" t="n"/>
-      <c r="D55" s="20" t="n"/>
+      <c r="A55" s="20" t="n"/>
+      <c r="B55" s="21" t="n"/>
+      <c r="C55" s="22" t="n"/>
+      <c r="D55" s="21" t="n"/>
     </row>
     <row r="56">
-      <c r="A56" s="19" t="n"/>
-      <c r="B56" s="20" t="n"/>
-      <c r="C56" s="21" t="n"/>
-      <c r="D56" s="20" t="n"/>
+      <c r="A56" s="20" t="n"/>
+      <c r="B56" s="21" t="n"/>
+      <c r="C56" s="22" t="n"/>
+      <c r="D56" s="21" t="n"/>
     </row>
     <row r="57">
-      <c r="A57" s="19" t="n"/>
-      <c r="B57" s="20" t="n"/>
-      <c r="C57" s="21" t="n"/>
-      <c r="D57" s="20" t="n"/>
+      <c r="A57" s="20" t="n"/>
+      <c r="B57" s="21" t="n"/>
+      <c r="C57" s="22" t="n"/>
+      <c r="D57" s="21" t="n"/>
     </row>
     <row r="58">
-      <c r="A58" s="19" t="n"/>
-      <c r="B58" s="20" t="n"/>
-      <c r="C58" s="21" t="n"/>
-      <c r="D58" s="20" t="n"/>
+      <c r="A58" s="20" t="n"/>
+      <c r="B58" s="21" t="n"/>
+      <c r="C58" s="22" t="n"/>
+      <c r="D58" s="21" t="n"/>
     </row>
     <row r="59">
-      <c r="A59" s="19" t="n"/>
-      <c r="B59" s="20" t="n"/>
-      <c r="C59" s="21" t="n"/>
-      <c r="D59" s="20" t="n"/>
+      <c r="A59" s="20" t="n"/>
+      <c r="B59" s="21" t="n"/>
+      <c r="C59" s="22" t="n"/>
+      <c r="D59" s="21" t="n"/>
     </row>
     <row r="60">
-      <c r="A60" s="19" t="n"/>
-      <c r="B60" s="20" t="n"/>
-      <c r="C60" s="21" t="n"/>
-      <c r="D60" s="20" t="n"/>
+      <c r="A60" s="20" t="n"/>
+      <c r="B60" s="21" t="n"/>
+      <c r="C60" s="22" t="n"/>
+      <c r="D60" s="21" t="n"/>
     </row>
     <row r="61">
-      <c r="A61" s="19" t="n"/>
-      <c r="B61" s="20" t="n"/>
-      <c r="C61" s="21" t="n"/>
-      <c r="D61" s="20" t="n"/>
+      <c r="A61" s="20" t="n"/>
+      <c r="B61" s="21" t="n"/>
+      <c r="C61" s="22" t="n"/>
+      <c r="D61" s="21" t="n"/>
     </row>
   </sheetData>
   <dataValidations count="2">
@@ -2211,86 +2238,86 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="22" t="inlineStr">
+      <c r="A1" s="23" t="inlineStr">
         <is>
           <t>How this ledger works</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="23" t="inlineStr"/>
+      <c r="A2" s="24" t="inlineStr"/>
     </row>
     <row r="3">
-      <c r="A3" s="23" t="inlineStr">
+      <c r="A3" s="24" t="inlineStr">
         <is>
           <t>MEMBERS: open the Ledger tab. It shows the total collected, how many people have given, and each person's total. Nothing on it can be typed into.</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="23" t="inlineStr"/>
+      <c r="A4" s="24" t="inlineStr"/>
     </row>
     <row r="5">
-      <c r="A5" s="23" t="inlineStr">
+      <c r="A5" s="24" t="inlineStr">
         <is>
           <t>MANAGER (Charles Quaye): open the Contributions tab and type one row per payment received:</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="23" t="inlineStr">
+      <c r="A6" s="24" t="inlineStr">
         <is>
           <t xml:space="preserve">   1. Date received – the day the money arrived.</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="23" t="inlineStr">
+      <c r="A7" s="24" t="inlineStr">
         <is>
           <t xml:space="preserve">   2. Member name – type the name the same way each time so the person's payments add up together (e.g. always 'Ama Mensah', not sometimes 'Ama').</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="23" t="inlineStr">
+      <c r="A8" s="24" t="inlineStr">
         <is>
           <t xml:space="preserve">   3. Amount (GHS) – the amount in cedis, numbers only.</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="23" t="inlineStr">
+      <c r="A9" s="24" t="inlineStr">
         <is>
           <t xml:space="preserve">   4. Note – optional. For money from abroad, put the original amount here, e.g. 'USD 50 via Western Union'.</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="23" t="inlineStr">
+      <c r="A10" s="24" t="inlineStr">
         <is>
           <t>The Ledger tab updates itself the moment a row is saved.</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="23" t="inlineStr"/>
+      <c r="A11" s="24" t="inlineStr"/>
     </row>
     <row r="12">
-      <c r="A12" s="23" t="inlineStr">
+      <c r="A12" s="24" t="inlineStr">
         <is>
           <t>The yellow cells with blue text are the ones to type in. Start on row 2, directly under the headings.</t>
         </is>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="23" t="inlineStr">
+      <c r="A13" s="24" t="inlineStr">
         <is>
           <t>To correct a mistake, edit the row. To remove a payment, clear the whole row.</t>
         </is>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="23" t="inlineStr">
+      <c r="A14" s="24" t="inlineStr">
         <is>
           <t>The Ledger tab lists up to 60 different contributors; payments themselves are unlimited.</t>
         </is>

</xml_diff>